<commit_message>
Added a script to automatically export a longitudinal profile for a given load case.
Use it by calling main_plot(). Comment out if unnecessary.
</commit_message>
<xml_diff>
--- a/Grammes/THL_Larisa/outputs/larisa2_2nd_submission_processed.xlsx
+++ b/Grammes/THL_Larisa/outputs/larisa2_2nd_submission_processed.xlsx
@@ -923,10 +923,10 @@
         <v>-71.73000000000002</v>
       </c>
       <c r="Q4" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R4" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S4" t="n">
         <v>7.767430340557276</v>
@@ -938,7 +938,7 @@
         <v>968.0528426736928</v>
       </c>
       <c r="V4" t="n">
-        <v>60.5</v>
+        <v>74.47</v>
       </c>
       <c r="W4" t="n">
         <v>3674.72694634428</v>
@@ -947,7 +947,7 @@
         <v>1004.850430705162</v>
       </c>
       <c r="Y4" t="n">
-        <v>62.8</v>
+        <v>77.3</v>
       </c>
       <c r="Z4" t="n">
         <v>4515.232134213278</v>
@@ -956,7 +956,7 @@
         <v>925.8990041527087</v>
       </c>
       <c r="AB4" t="n">
-        <v>79.36</v>
+        <v>97.67</v>
       </c>
       <c r="AC4" t="n">
         <v>4334.568258652236</v>
@@ -965,7 +965,7 @@
         <v>899.6579021198809</v>
       </c>
       <c r="AE4" t="n">
-        <v>77.11</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="AF4" t="n">
         <v>9.565584882570509</v>
@@ -977,7 +977,7 @@
         <v>789.1148714407962</v>
       </c>
       <c r="AI4" t="n">
-        <v>49.32</v>
+        <v>60.7</v>
       </c>
       <c r="AJ4" t="n">
         <v>0</v>
@@ -1060,10 +1060,10 @@
         <v>-111.08</v>
       </c>
       <c r="Q5" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R5" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S5" t="n">
         <v>16.1029295827366</v>
@@ -1075,7 +1075,7 @@
         <v>413.3076536509018</v>
       </c>
       <c r="V5" t="n">
-        <v>25.83</v>
+        <v>31.79</v>
       </c>
       <c r="W5" t="n">
         <v>3216.290344954967</v>
@@ -1084,7 +1084,7 @@
         <v>403.8470637126914</v>
       </c>
       <c r="Y5" t="n">
-        <v>25.24</v>
+        <v>31.07</v>
       </c>
       <c r="Z5" t="n">
         <v>4175.373701010977</v>
@@ -1093,7 +1093,7 @@
         <v>425.0760629898817</v>
       </c>
       <c r="AB5" t="n">
-        <v>36.43</v>
+        <v>44.84</v>
       </c>
       <c r="AC5" t="n">
         <v>4078.033859485204</v>
@@ -1102,7 +1102,7 @@
         <v>430.8694365724957</v>
       </c>
       <c r="AE5" t="n">
-        <v>36.93</v>
+        <v>45.45</v>
       </c>
       <c r="AF5" t="n">
         <v>18.06960183865581</v>
@@ -1114,7 +1114,7 @@
         <v>446.0720151564881</v>
       </c>
       <c r="AI5" t="n">
-        <v>27.88</v>
+        <v>34.31</v>
       </c>
       <c r="AJ5" t="n">
         <v>119.5245674354994</v>
@@ -1129,10 +1129,10 @@
         <v>0</v>
       </c>
       <c r="AN5" t="n">
-        <v>0</v>
+        <v>115.5408807666297</v>
       </c>
       <c r="AO5" t="n">
-        <v>0</v>
+        <v>72.91713076662967</v>
       </c>
     </row>
     <row r="6">
@@ -1862,10 +1862,10 @@
         <v>21.68000000000006</v>
       </c>
       <c r="Q11" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R11" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S11" t="n">
         <v>6.351345738596736</v>
@@ -1877,7 +1877,7 @@
         <v>759.7718759190915</v>
       </c>
       <c r="V11" t="n">
-        <v>47.49</v>
+        <v>58.44</v>
       </c>
       <c r="W11" t="n">
         <v>3675.82229884234</v>
@@ -1886,7 +1886,7 @@
         <v>781.1425697633979</v>
       </c>
       <c r="Y11" t="n">
-        <v>48.82</v>
+        <v>60.09</v>
       </c>
       <c r="Z11" t="n">
         <v>4453.051930597556</v>
@@ -1895,7 +1895,7 @@
         <v>735.6109981335308</v>
       </c>
       <c r="AB11" t="n">
-        <v>63.05</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AC11" t="n">
         <v>4252.102813957528</v>
@@ -1904,7 +1904,7 @@
         <v>719.8675967460401</v>
       </c>
       <c r="AE11" t="n">
-        <v>61.7</v>
+        <v>75.94</v>
       </c>
       <c r="AF11" t="n">
         <v>7.812285460757115</v>
@@ -1916,7 +1916,7 @@
         <v>646.2396636686643</v>
       </c>
       <c r="AI11" t="n">
-        <v>40.39</v>
+        <v>49.71</v>
       </c>
       <c r="AJ11" t="n">
         <v>0</v>
@@ -2394,10 +2394,10 @@
         <v>-69.06999999999999</v>
       </c>
       <c r="Q15" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R15" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S15" t="n">
         <v>6.28109898141342</v>
@@ -2409,7 +2409,7 @@
         <v>277.0477466246882</v>
       </c>
       <c r="V15" t="n">
-        <v>17.32</v>
+        <v>21.31</v>
       </c>
       <c r="W15" t="n">
         <v>952.6027824683442</v>
@@ -2418,7 +2418,7 @@
         <v>273.5054423718399</v>
       </c>
       <c r="Y15" t="n">
-        <v>17.09</v>
+        <v>21.04</v>
       </c>
       <c r="Z15" t="n">
         <v>1286.829842898191</v>
@@ -2427,7 +2427,7 @@
         <v>288.7791929070686</v>
       </c>
       <c r="AB15" t="n">
-        <v>24.75</v>
+        <v>30.46</v>
       </c>
       <c r="AC15" t="n">
         <v>1258.375987476826</v>
@@ -2436,7 +2436,7 @@
         <v>290.6686617707402</v>
       </c>
       <c r="AE15" t="n">
-        <v>24.91</v>
+        <v>30.66</v>
       </c>
       <c r="AF15" t="n">
         <v>7.02692901075106</v>
@@ -2448,7 +2448,7 @@
         <v>312.9407609517943</v>
       </c>
       <c r="AI15" t="n">
-        <v>19.56</v>
+        <v>24.07</v>
       </c>
       <c r="AJ15" t="n">
         <v>0</v>
@@ -2527,10 +2527,10 @@
         <v>-34.5</v>
       </c>
       <c r="Q16" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R16" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S16" t="n">
         <v>44.46846285253827</v>
@@ -2542,7 +2542,7 @@
         <v>314.1464498201202</v>
       </c>
       <c r="V16" t="n">
-        <v>19.63</v>
+        <v>24.17</v>
       </c>
       <c r="W16" t="n">
         <v>2925.135112433156</v>
@@ -2551,7 +2551,7 @@
         <v>309.8240820884087</v>
       </c>
       <c r="Y16" t="n">
-        <v>19.36</v>
+        <v>23.83</v>
       </c>
       <c r="Z16" t="n">
         <v>3933.835847641682</v>
@@ -2560,7 +2560,7 @@
         <v>311.6727637802096</v>
       </c>
       <c r="AB16" t="n">
-        <v>26.71</v>
+        <v>32.88</v>
       </c>
       <c r="AC16" t="n">
         <v>3896.556419877462</v>
@@ -2569,7 +2569,7 @@
         <v>315.7712789867284</v>
       </c>
       <c r="AE16" t="n">
-        <v>27.06</v>
+        <v>33.31</v>
       </c>
       <c r="AF16" t="n">
         <v>46.53197425332766</v>
@@ -2581,7 +2581,7 @@
         <v>328.942899661527</v>
       </c>
       <c r="AI16" t="n">
-        <v>20.56</v>
+        <v>25.3</v>
       </c>
       <c r="AJ16" t="n">
         <v>110.5083932321411</v>
@@ -2596,10 +2596,10 @@
         <v>0</v>
       </c>
       <c r="AN16" t="n">
-        <v>0</v>
+        <v>68.24203089581245</v>
       </c>
       <c r="AO16" t="n">
-        <v>0</v>
+        <v>25.61828089581245</v>
       </c>
     </row>
     <row r="17">
@@ -2660,10 +2660,10 @@
         <v>102.7599999999999</v>
       </c>
       <c r="Q17" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R17" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S17" t="n">
         <v>14.38553588035727</v>
@@ -2675,7 +2675,7 @@
         <v>215.2657232396864</v>
       </c>
       <c r="V17" t="n">
-        <v>13.45</v>
+        <v>16.56</v>
       </c>
       <c r="W17" t="n">
         <v>926.1666820088807</v>
@@ -2684,7 +2684,7 @@
         <v>212.3546133876593</v>
       </c>
       <c r="Y17" t="n">
-        <v>13.27</v>
+        <v>16.33</v>
       </c>
       <c r="Z17" t="n">
         <v>1261.948052365319</v>
@@ -2693,7 +2693,7 @@
         <v>215.1655617505313</v>
       </c>
       <c r="AB17" t="n">
-        <v>18.44</v>
+        <v>22.7</v>
       </c>
       <c r="AC17" t="n">
         <v>1249.356387857644</v>
@@ -2702,7 +2702,7 @@
         <v>217.971757206723</v>
       </c>
       <c r="AE17" t="n">
-        <v>18.68</v>
+        <v>22.99</v>
       </c>
       <c r="AF17" t="n">
         <v>15.03620736057636</v>
@@ -2714,7 +2714,7 @@
         <v>232.2373656166178</v>
       </c>
       <c r="AI17" t="n">
-        <v>14.51</v>
+        <v>17.86</v>
       </c>
       <c r="AJ17" t="n">
         <v>0</v>
@@ -2793,10 +2793,10 @@
         <v>-35.16999999999996</v>
       </c>
       <c r="Q18" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R18" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S18" t="n">
         <v>10.95579855709367</v>
@@ -2808,7 +2808,7 @@
         <v>686.079152291356</v>
       </c>
       <c r="V18" t="n">
-        <v>42.88</v>
+        <v>52.78</v>
       </c>
       <c r="W18" t="n">
         <v>3433.637380599765</v>
@@ -2817,7 +2817,7 @@
         <v>694.4787645163276</v>
       </c>
       <c r="Y18" t="n">
-        <v>43.4</v>
+        <v>53.42</v>
       </c>
       <c r="Z18" t="n">
         <v>4344.952342031889</v>
@@ -2826,7 +2826,7 @@
         <v>680.2525969234546</v>
       </c>
       <c r="AB18" t="n">
-        <v>58.3</v>
+        <v>71.76000000000001</v>
       </c>
       <c r="AC18" t="n">
         <v>4207.844108633339</v>
@@ -2835,7 +2835,7 @@
         <v>673.2927131884063</v>
       </c>
       <c r="AE18" t="n">
-        <v>57.71</v>
+        <v>71.03</v>
       </c>
       <c r="AF18" t="n">
         <v>12.89559873051838</v>
@@ -2847,7 +2847,7 @@
         <v>642.1215368149512</v>
       </c>
       <c r="AI18" t="n">
-        <v>40.13</v>
+        <v>49.39</v>
       </c>
       <c r="AJ18" t="n">
         <v>0</v>
@@ -3325,10 +3325,10 @@
         <v>-84.38</v>
       </c>
       <c r="Q22" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R22" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S22" t="n">
         <v>9.624423503362092</v>
@@ -3340,7 +3340,7 @@
         <v>851.2352914619994</v>
       </c>
       <c r="V22" t="n">
-        <v>53.2</v>
+        <v>65.48</v>
       </c>
       <c r="W22" t="n">
         <v>3524.39321032992</v>
@@ -3349,7 +3349,7 @@
         <v>881.5834693287155</v>
       </c>
       <c r="Y22" t="n">
-        <v>55.1</v>
+        <v>67.81</v>
       </c>
       <c r="Z22" t="n">
         <v>4412.915496547596</v>
@@ -3358,7 +3358,7 @@
         <v>819.0840610596792</v>
       </c>
       <c r="AB22" t="n">
-        <v>70.2</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AC22" t="n">
         <v>4259.958789734415</v>
@@ -3367,7 +3367,7 @@
         <v>797.1846706146812</v>
       </c>
       <c r="AE22" t="n">
-        <v>68.33</v>
+        <v>84.09</v>
       </c>
       <c r="AF22" t="n">
         <v>11.55568860923826</v>
@@ -3379,7 +3379,7 @@
         <v>718.2838802084441</v>
       </c>
       <c r="AI22" t="n">
-        <v>44.89</v>
+        <v>55.25</v>
       </c>
       <c r="AJ22" t="n">
         <v>0</v>
@@ -3595,10 +3595,10 @@
         <v>-73.03000000000003</v>
       </c>
       <c r="Q24" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R24" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S24" t="n">
         <v>3.204554385964912</v>
@@ -3610,7 +3610,7 @@
         <v>1028.742046033204</v>
       </c>
       <c r="V24" t="n">
-        <v>64.3</v>
+        <v>79.13</v>
       </c>
       <c r="W24" t="n">
         <v>3772.660197771894</v>
@@ -3619,7 +3619,7 @@
         <v>1083.661882151806</v>
       </c>
       <c r="Y24" t="n">
-        <v>67.73</v>
+        <v>83.36</v>
       </c>
       <c r="Z24" t="n">
         <v>4334.087508189165</v>
@@ -3628,7 +3628,7 @@
         <v>972.5848128424816</v>
       </c>
       <c r="AB24" t="n">
-        <v>83.36</v>
+        <v>102.6</v>
       </c>
       <c r="AC24" t="n">
         <v>4056.875184437656</v>
@@ -3637,7 +3637,7 @@
         <v>935.7527637918256</v>
       </c>
       <c r="AE24" t="n">
-        <v>80.2</v>
+        <v>98.70999999999999</v>
       </c>
       <c r="AF24" t="n">
         <v>3.927741351072034</v>
@@ -3649,7 +3649,7 @@
         <v>864.8903527212537</v>
       </c>
       <c r="AI24" t="n">
-        <v>54.06</v>
+        <v>66.53</v>
       </c>
       <c r="AJ24" t="n">
         <v>0</v>
@@ -4272,10 +4272,10 @@
         <v>-42.79000000000002</v>
       </c>
       <c r="Q29" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R29" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S29" t="n">
         <v>4.676978789304928</v>
@@ -4287,7 +4287,7 @@
         <v>999.3275698831206</v>
       </c>
       <c r="V29" t="n">
-        <v>62.46</v>
+        <v>76.87</v>
       </c>
       <c r="W29" t="n">
         <v>3717.870086030118</v>
@@ -4296,7 +4296,7 @@
         <v>1064.152912363578</v>
       </c>
       <c r="Y29" t="n">
-        <v>66.51000000000001</v>
+        <v>81.86</v>
       </c>
       <c r="Z29" t="n">
         <v>4400.824365789411</v>
@@ -4305,7 +4305,7 @@
         <v>932.7606722778983</v>
       </c>
       <c r="AB29" t="n">
-        <v>79.95</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AC29" t="n">
         <v>4166.819345815501</v>
@@ -4314,7 +4314,7 @@
         <v>889.2341144133447</v>
       </c>
       <c r="AE29" t="n">
-        <v>76.22</v>
+        <v>93.81</v>
       </c>
       <c r="AF29" t="n">
         <v>5.686382476376037</v>
@@ -4326,7 +4326,7 @@
         <v>804.1155962871071</v>
       </c>
       <c r="AI29" t="n">
-        <v>50.26</v>
+        <v>61.86</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -5074,10 +5074,10 @@
         <v>-56.62</v>
       </c>
       <c r="Q35" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R35" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S35" t="n">
         <v>18.10874719194247</v>
@@ -5089,7 +5089,7 @@
         <v>942.113204322744</v>
       </c>
       <c r="V35" t="n">
-        <v>58.88</v>
+        <v>72.47</v>
       </c>
       <c r="W35" t="n">
         <v>3561.574931652337</v>
@@ -5098,7 +5098,7 @@
         <v>982.3394376528789</v>
       </c>
       <c r="Y35" t="n">
-        <v>61.4</v>
+        <v>75.56</v>
       </c>
       <c r="Z35" t="n">
         <v>4607.249881015574</v>
@@ -5107,7 +5107,7 @@
         <v>900.2791042895162</v>
       </c>
       <c r="AB35" t="n">
-        <v>77.16</v>
+        <v>94.97</v>
       </c>
       <c r="AC35" t="n">
         <v>4503.973921780856</v>
@@ -5116,7 +5116,7 @@
         <v>872.7443475373484</v>
       </c>
       <c r="AE35" t="n">
-        <v>74.8</v>
+        <v>92.06999999999999</v>
       </c>
       <c r="AF35" t="n">
         <v>21.63268387675932</v>
@@ -5128,7 +5128,7 @@
         <v>794.4354411498384</v>
       </c>
       <c r="AI35" t="n">
-        <v>49.65</v>
+        <v>61.11</v>
       </c>
       <c r="AJ35" t="n">
         <v>0</v>
@@ -8270,10 +8270,10 @@
         <v>-35.31</v>
       </c>
       <c r="Q59" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R59" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S59" t="n">
         <v>2.389124924174844</v>
@@ -8285,7 +8285,7 @@
         <v>1099.204696707569</v>
       </c>
       <c r="V59" t="n">
-        <v>68.7</v>
+        <v>84.55</v>
       </c>
       <c r="W59" t="n">
         <v>3813.013819252533</v>
@@ -8294,7 +8294,7 @@
         <v>1182.599231821315</v>
       </c>
       <c r="Y59" t="n">
-        <v>73.91</v>
+        <v>90.97</v>
       </c>
       <c r="Z59" t="n">
         <v>4284.95974443958</v>
@@ -8303,7 +8303,7 @@
         <v>1014.588142449815</v>
       </c>
       <c r="AB59" t="n">
-        <v>86.95999999999999</v>
+        <v>107.03</v>
       </c>
       <c r="AC59" t="n">
         <v>3974.729626829252</v>
@@ -8312,7 +8312,7 @@
         <v>959.2550801958007</v>
       </c>
       <c r="AE59" t="n">
-        <v>82.22</v>
+        <v>101.19</v>
       </c>
       <c r="AF59" t="n">
         <v>2.912071051958794</v>
@@ -8324,7 +8324,7 @@
         <v>870.2515998645058</v>
       </c>
       <c r="AI59" t="n">
-        <v>54.39</v>
+        <v>66.94</v>
       </c>
       <c r="AJ59" t="n">
         <v>0</v>
@@ -10668,10 +10668,10 @@
         <v>-89.69000000000003</v>
       </c>
       <c r="Q77" t="n">
-        <v>1600</v>
+        <v>1300</v>
       </c>
       <c r="R77" t="n">
-        <v>5833.599999999999</v>
+        <v>4739.8</v>
       </c>
       <c r="S77" t="n">
         <v>7.767430340557276</v>
@@ -10683,7 +10683,7 @@
         <v>589.495458577133</v>
       </c>
       <c r="V77" t="n">
-        <v>36.84</v>
+        <v>45.35</v>
       </c>
       <c r="W77" t="n">
         <v>3674.72694634428</v>
@@ -10692,7 +10692,7 @@
         <v>599.8203321958699</v>
       </c>
       <c r="Y77" t="n">
-        <v>37.49</v>
+        <v>46.14</v>
       </c>
       <c r="Z77" t="n">
         <v>4515.232134213278</v>
@@ -10701,7 +10701,7 @@
         <v>576.8794621593414</v>
       </c>
       <c r="AB77" t="n">
-        <v>49.44</v>
+        <v>60.85</v>
       </c>
       <c r="AC77" t="n">
         <v>4334.568258652236</v>
@@ -10710,7 +10710,7 @@
         <v>568.6448459377145</v>
       </c>
       <c r="AE77" t="n">
-        <v>48.74</v>
+        <v>59.99</v>
       </c>
       <c r="AF77" t="n">
         <v>9.565584882570509</v>
@@ -10722,7 +10722,7 @@
         <v>513.1375488788611</v>
       </c>
       <c r="AI77" t="n">
-        <v>32.07</v>
+        <v>39.47</v>
       </c>
       <c r="AJ77" t="n">
         <v>23.08986009426201</v>

</xml_diff>